<commit_message>
model number for 27P changed from vx156620 to vx155480 and some zpl code from VX.. to VQ..
</commit_message>
<xml_diff>
--- a/models/hv/data/bms_scan_log.xlsx
+++ b/models/hv/data/bms_scan_log.xlsx
@@ -1,101 +1,43 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RadarCalibration\Desktop\hv_only_project\bms_label_suite\models\hv\data\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B288E1C-D4E3-495D-8802-037BE5741A04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="bmb_cmb" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="bmb_cmb" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
-  <si>
-    <t>Sl.No</t>
-  </si>
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>Time</t>
-  </si>
-  <si>
-    <t>Pack QR Data</t>
-  </si>
-  <si>
-    <t>BMB ID</t>
-  </si>
-  <si>
-    <t>CMB ID</t>
-  </si>
-  <si>
-    <t>Rework BMB ID</t>
-  </si>
-  <si>
-    <t>Rework CMB ID</t>
-  </si>
-  <si>
-    <t>28 May 2026</t>
-  </si>
-  <si>
-    <t>2:23:44 PM</t>
-  </si>
-  <si>
-    <t>VX155800:ABA61202605281A00114</t>
-  </si>
-  <si>
-    <t>VQ150720_1.0X26030083</t>
-  </si>
-  <si>
-    <t>VQ150710-REV-A-S26250069</t>
-  </si>
-  <si>
-    <t>03 Aug 2026</t>
-  </si>
-  <si>
-    <t>1:09:20 PM</t>
-  </si>
-  <si>
-    <t>VX156070:ABA41202608031A00130</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="3">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Segoe UI"/>
     </font>
     <font>
+      <name val="Segoe UI"/>
       <sz val="10"/>
-      <name val="Segoe UI"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -108,6 +50,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFEEF2F7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EEF2F7"/>
       </patternFill>
     </fill>
   </fills>
@@ -123,37 +70,102 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+  <cellXfs count="8">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -441,86 +453,158 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="7" customWidth="1"/>
-    <col min="2" max="2" width="13" customWidth="1"/>
-    <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="40" customWidth="1"/>
-    <col min="5" max="8" width="26" customWidth="1"/>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+    <row r="1" ht="28.05" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Sl.No</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Pack QR Data</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>BMB ID</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>CMB ID</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Rework BMB ID</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Rework CMB ID</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>2:23:44 PM</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>VX155800:ABA61202605281A00114</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>VQ150720_1.0X26030083</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>VQ150710-REV-A-S26250069</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="n"/>
+      <c r="H2" s="3" t="n"/>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>03 Aug 2026</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>1:09:20 PM</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>VX156070:ABA41202608031A00130</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>VQ150720_1.0X26030083</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>VQ150710-REV-A-S26250069</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="n"/>
+      <c r="H3" s="5" t="n"/>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="2">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-    </row>
-    <row r="3" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="4">
-        <v>2</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G3" s="5"/>
-      <c r="H3" s="5"/>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>2:27:49 PM</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>VX156080:ABA31202605281A00119</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>VQ150720-REV-A-S26250069</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>VQ150710-2V2S26250088</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
resequencing of sl.no is updated for .csv files
</commit_message>
<xml_diff>
--- a/models/hv/data/bms_scan_log.xlsx
+++ b/models/hv/data/bms_scan_log.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="bmb_cmb" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="bmb_cmb" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -70,7 +70,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -92,6 +92,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -458,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -638,6 +641,46 @@
       <c r="G5" s="5" t="inlineStr"/>
       <c r="H5" s="5" t="inlineStr"/>
     </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>04:28:55 PM</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U00108</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>VQ150720-REV-A-S26250069</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>VQ150710-2V2S26250088</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>VQ150720-REV-A-S26250061</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>VQ150710-2V2S26250082</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
added api keys with toggle to enable and validate them, and added machine_ details to ui
</commit_message>
<xml_diff>
--- a/models/hv/data/bms_scan_log.xlsx
+++ b/models/hv/data/bms_scan_log.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="bmb_cmb" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="bmb_cmb" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -681,6 +681,38 @@
         </is>
       </c>
     </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>08:44:10 AM</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U00118</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>VQ150720_1.0X26030083</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>VQ150710-2V2S26250082</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
machine details updated for battery pack dummy id too
</commit_message>
<xml_diff>
--- a/models/hv/data/bms_scan_log.xlsx
+++ b/models/hv/data/bms_scan_log.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,8 +34,14 @@
       <name val="Segoe UI"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -57,6 +63,11 @@
         <fgColor rgb="00EEF2F7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -70,7 +81,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -95,6 +106,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -461,17 +475,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <dimension ref="A1:J8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" outlineLevelCol="0"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
     <col width="26" customWidth="1" min="5" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28.05" customHeight="1">
+    <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Sl.No</t>
@@ -510,6 +526,16 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Rework CMB ID</t>
+        </is>
+      </c>
+      <c r="I1" s="9" t="inlineStr">
+        <is>
+          <t>Machine Name</t>
+        </is>
+      </c>
+      <c r="J1" s="9" t="inlineStr">
+        <is>
+          <t>Machine ID</t>
         </is>
       </c>
     </row>
@@ -713,6 +739,48 @@
       <c r="G7" s="5" t="inlineStr"/>
       <c r="H7" s="5" t="inlineStr"/>
     </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>01:37:33 PM</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U00134</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>VQ150720_1.0X26030083</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>VQ150710-2V2S26250082</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr"/>
+      <c r="H8" s="7" t="inlineStr"/>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>pc_2</t>
+        </is>
+      </c>
+      <c r="J8" s="6" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
bms rework approach changed, removed patch from client server side, aligned misconfigured variables in gui
</commit_message>
<xml_diff>
--- a/models/hv/data/bms_scan_log.xlsx
+++ b/models/hv/data/bms_scan_log.xlsx
@@ -2,14 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="bmb_cmb" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -27,7 +28,7 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
@@ -36,12 +37,11 @@
     </font>
     <font>
       <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FF0000FF"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -50,22 +50,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1F3864"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEEF2F7"/>
+        <fgColor rgb="001F3864"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00EEF2F7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001F3864"/>
       </patternFill>
     </fill>
   </fills>
@@ -81,7 +71,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -98,21 +88,12 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -475,16 +456,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" outlineLevelCol="0"/>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -520,20 +503,15 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Rework BMB ID</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Rework CMB ID</t>
-        </is>
-      </c>
-      <c r="I1" s="9" t="inlineStr">
-        <is>
           <t>Machine Name</t>
         </is>
       </c>
-      <c r="J1" s="9" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Machine ID</t>
         </is>
@@ -545,31 +523,36 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>28 May 2026</t>
+          <t>24 Sep 2026</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>2:23:44 PM</t>
+          <t>09:12:16 AM</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>VX155800:ABA61202605281A00114</t>
+          <t>VQ150000:ABA31202609241R00295</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>VQ150720_1.0X26030083</t>
+          <t>VQ150720-REV-A-S26250061</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>VQ150710-REV-A-S26250069</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="n"/>
-      <c r="H2" s="3" t="n"/>
+          <t>VQ150710-2V2S26250082</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr"/>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="4" t="n">
@@ -577,63 +560,81 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>03 Aug 2026</t>
+          <t>24 Sep 2026</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>1:09:20 PM</t>
+          <t>09:13:19 AM</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>VX156070:ABA41202608031A00130</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
+          <t>VQ150000:ABA31202609241R00295</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>VQ150720_1.0X26030083</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>VQ150710-REV-A-S26250069</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="n"/>
-      <c r="H3" s="5" t="n"/>
+          <t>VQ150710-2V2S26250082</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>Rework 1</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr"/>
+      <c r="I3" s="4" t="inlineStr"/>
     </row>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="6" t="n">
+      <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>28 May 2026</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>2:27:49 PM</t>
-        </is>
-      </c>
-      <c r="D4" s="7" t="inlineStr">
-        <is>
-          <t>VX156080:ABA31202605281A00119</t>
-        </is>
-      </c>
-      <c r="E4" s="7" t="inlineStr">
-        <is>
-          <t>VQ150720-REV-A-S26250069</t>
-        </is>
-      </c>
-      <c r="F4" s="7" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>24 Sep 2026</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>09:18:06 AM</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>VQ150000:ABA31202609241R00295</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>VQ150720_1.0X26030086</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>VQ150710-2V2S26250088</t>
         </is>
       </c>
-      <c r="G4" s="7" t="inlineStr"/>
-      <c r="H4" s="7" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="4" t="n">
@@ -641,22 +642,22 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>28 May 2026</t>
+          <t>24 Sep 2026</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>8:35:03 AM</t>
+          <t>09:19:17 AM</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>VX156060:ABA51202605281U00111</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>VQ150720-REV-A-S26250069</t>
+          <t>VQ150000:ABA31202609241R00295</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>VQ150720-REV-A-S26250064</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
@@ -664,120 +665,19 @@
           <t>VQ150710-2V2S26250088</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr"/>
-    </row>
-    <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>28 May 2026</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>04:28:55 PM</t>
-        </is>
-      </c>
-      <c r="D6" s="7" t="inlineStr">
-        <is>
-          <t>VX156060:ABA51202605281U00108</t>
-        </is>
-      </c>
-      <c r="E6" s="7" t="inlineStr">
-        <is>
-          <t>VQ150720-REV-A-S26250069</t>
-        </is>
-      </c>
-      <c r="F6" s="7" t="inlineStr">
-        <is>
-          <t>VQ150710-2V2S26250088</t>
-        </is>
-      </c>
-      <c r="G6" s="8" t="inlineStr">
-        <is>
-          <t>VQ150720-REV-A-S26250061</t>
-        </is>
-      </c>
-      <c r="H6" s="8" t="inlineStr">
-        <is>
-          <t>VQ150710-2V2S26250082</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>28 May 2026</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>08:44:10 AM</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>VX156060:ABA51202605281U00118</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>VQ150720_1.0X26030083</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>VQ150710-2V2S26250082</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr"/>
-    </row>
-    <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>28 May 2026</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>01:37:33 PM</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>VX156060:ABA51202605281U00134</t>
-        </is>
-      </c>
-      <c r="E8" s="7" t="inlineStr">
-        <is>
-          <t>VQ150720_1.0X26030083</t>
-        </is>
-      </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>VQ150710-2V2S26250082</t>
-        </is>
-      </c>
-      <c r="G8" s="7" t="inlineStr"/>
-      <c r="H8" s="7" t="inlineStr"/>
-      <c r="I8" s="6" t="inlineStr">
-        <is>
-          <t>pc_2</t>
-        </is>
-      </c>
-      <c r="J8" s="6" t="inlineStr">
-        <is>
-          <t>M2</t>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Rework 2</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
zpl and label.py code optimized and removed unnecessary and unused code snippet
</commit_message>
<xml_diff>
--- a/models/hv/data/bms_scan_log.xlsx
+++ b/models/hv/data/bms_scan_log.xlsx
@@ -71,7 +71,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -89,6 +89,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -456,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -681,6 +684,154 @@
         </is>
       </c>
     </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>10:49:11 AM</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U00139</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>VQ150720_1.0X26030086</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>VQ150710-2V2S26250088</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>10:52:03 AM</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U00139</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>VQ150720-REV-A-S26250064</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>VQ150710-2V2S26250088</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr"/>
+      <c r="I7" s="4" t="inlineStr"/>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>10:53:40 AM</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U00139</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>VQ150720-REV-A-S26250064</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>VQ150710-2V2S26250089</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Rework 1</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>29 Sep 2026</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>02:46:49 PM</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>VQ150010:ABA41202609292R00309</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>VQ150720-REV-A-S26250064</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>VQ150710-2V2S26250088</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr"/>
+      <c r="I9" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
serial_count and api parameters unauthorized issues are corrected, stepr.txt file updated to add further battery parameters
</commit_message>
<xml_diff>
--- a/models/hv/data/bms_scan_log.xlsx
+++ b/models/hv/data/bms_scan_log.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -832,6 +832,51 @@
       <c r="H9" s="4" t="inlineStr"/>
       <c r="I9" s="4" t="inlineStr"/>
     </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>30 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>12:32:53 PM</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>BP00000131:ADT11202610301R00006</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>VQ150720_1.0X26030086</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>VQ150710-2V2S26250088</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>